<commit_message>
Added funtionality to edit the patrols
</commit_message>
<xml_diff>
--- a/docs/samples/weekly-roster-template.xlsx
+++ b/docs/samples/weekly-roster-template.xlsx
@@ -68,7 +68,7 @@
     <t>3.</t>
   </si>
   <si>
-    <t>Both people must be registered, active users at the same location. The email has to match their account exactly.</t>
+    <t>Both people must be registered, active users at the same location. The EHS Officer may enter their own email, as an auditor or an auditee. The email has to match their account exactly.</t>
   </si>
   <si>
     <t>4.</t>
@@ -101,7 +101,7 @@
     <t>If any row has a problem, nothing is saved and every problem is listed with its row number, so fix them and upload again.</t>
   </si>
   <si>
-    <t>Afterwards you can still change the auditor or auditee for a zone from the dashboard, and the change applies to every remaining Monday of the year.</t>
+    <t>Afterwards you can change a zone's auditor or auditee from the dashboard, for every remaining audit of the year or for a single week. Uploading the roster again overwrites those changes with what the file says.</t>
   </si>
 </sst>
 </file>
@@ -606,7 +606,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -725,6 +725,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>